<commit_message>
Make job apply links visible as full URLs in Jobs tab
Display the full posting URL as clickable text in the Apply Link column
(was a hidden 'Apply arrow' label) and widen the column so every link is
readable and copyable.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RE7NV69kCeMfgUMKPAdCCj
</commit_message>
<xml_diff>
--- a/David_StJulus_Job_Search_Tracker.xlsx
+++ b/David_StJulus_Job_Search_Tracker.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="952" uniqueCount="495">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="952" uniqueCount="544">
   <si>
     <t xml:space="preserve">JOB SEARCH  COMMAND  CENTER</t>
   </si>
@@ -277,7 +277,7 @@
     <t xml:space="preserve">$18–$23/hr</t>
   </si>
   <si>
-    <t xml:space="preserve">Apply ↗</t>
+    <t xml:space="preserve">https://to.indeed.com/aax99gw6hbrb</t>
   </si>
   <si>
     <t xml:space="preserve">Direct QBO bookkeeping match — your core daily tool</t>
@@ -301,6 +301,9 @@
     <t xml:space="preserve">$25–$30/hr</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aay7xrszvfcz</t>
+  </si>
+  <si>
     <t xml:space="preserve">Full-charge bookkeeping for a local firm; multi-client like your current work</t>
   </si>
   <si>
@@ -319,6 +322,9 @@
     <t xml:space="preserve">$65,000–$70,000</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aavpsvxl96nc</t>
+  </si>
+  <si>
     <t xml:space="preserve">Combined bookkeeping + staff accounting — fits your hybrid skill set</t>
   </si>
   <si>
@@ -331,6 +337,9 @@
     <t xml:space="preserve">$58,380–$70,307</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aa7fjmb4wpj2</t>
+  </si>
+  <si>
     <t xml:space="preserve">Entry/junior accountant role — reconciliations and journal entries</t>
   </si>
   <si>
@@ -346,6 +355,9 @@
     <t xml:space="preserve">$30–$35/hr</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aacwsr2qtwlb</t>
+  </si>
+  <si>
     <t xml:space="preserve">Classic staff accountant duties matching your full-cycle experience</t>
   </si>
   <si>
@@ -361,6 +373,9 @@
     <t xml:space="preserve">$50,000–$60,000</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aal4dgvq6xv9</t>
+  </si>
+  <si>
     <t xml:space="preserve">Job-cost accounting; builds on your profitability/unit-economics work</t>
   </si>
   <si>
@@ -379,6 +394,9 @@
     <t xml:space="preserve">$62,000–$75,000</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aajvsvfvjwrc</t>
+  </si>
+  <si>
     <t xml:space="preserve">Full-charge bookkeeping for a small business — your sweet spot</t>
   </si>
   <si>
@@ -397,6 +415,9 @@
     <t xml:space="preserve">$20–$29/hr</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aaps72t8dk8f</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bookkeeping support role, easy entry near Manchester</t>
   </si>
   <si>
@@ -415,6 +436,9 @@
     <t xml:space="preserve">$58,000–$66,000</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aa2qxtmxy4bd</t>
+  </si>
+  <si>
     <t xml:space="preserve">Full accounting admin for a small firm; QBO/Excel focused</t>
   </si>
   <si>
@@ -433,6 +457,9 @@
     <t xml:space="preserve">$54,930–$87,662</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aads28mmkhyq</t>
+  </si>
+  <si>
     <t xml:space="preserve">Full-charge bookkeeping with strong pay range</t>
   </si>
   <si>
@@ -451,6 +478,9 @@
     <t xml:space="preserve">N/A</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aa7g6jc9nyk9</t>
+  </si>
+  <si>
     <t xml:space="preserve">Dealership accounting office — transaction-heavy reconciliation work</t>
   </si>
   <si>
@@ -469,6 +499,9 @@
     <t xml:space="preserve">$60,000–$70,000</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aavdnzl4qqkf</t>
+  </si>
+  <si>
     <t xml:space="preserve">Finance operations + reporting; mirrors your fractional-CFO duties</t>
   </si>
   <si>
@@ -484,6 +517,9 @@
     <t xml:space="preserve">$22–$25/hr</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aa7r9mwd7n4z</t>
+  </si>
+  <si>
     <t xml:space="preserve">Local Manchester accounting support role — short commute</t>
   </si>
   <si>
@@ -499,6 +535,9 @@
     <t xml:space="preserve">$75,000–$90,000</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aay7qpqwv4hm</t>
+  </si>
+  <si>
     <t xml:space="preserve">FP&amp;A role matching your KPI dashboards, budgeting &amp; forecasting</t>
   </si>
   <si>
@@ -514,6 +553,9 @@
     <t xml:space="preserve">From $40/hr</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aajzj8rzxsjj</t>
+  </si>
+  <si>
     <t xml:space="preserve">Part-time accounting leadership; fits fractional/multi-client style</t>
   </si>
   <si>
@@ -532,6 +574,9 @@
     <t xml:space="preserve">$29.05–$36.26/hr</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aaygkdv8pht9</t>
+  </si>
+  <si>
     <t xml:space="preserve">Municipal finance; stable role using reconciliations &amp; reporting</t>
   </si>
   <si>
@@ -547,6 +592,9 @@
     <t xml:space="preserve">$64,000–$78,000</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aa4gbvpbhrlr</t>
+  </si>
+  <si>
     <t xml:space="preserve">Senior accountant role; reporting-heavy, solid pay</t>
   </si>
   <si>
@@ -562,6 +610,9 @@
     <t xml:space="preserve">$80,000–$90,000</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aabjzr679tlv</t>
+  </si>
+  <si>
     <t xml:space="preserve">Senior accountant with month-end close — aim-higher option</t>
   </si>
   <si>
@@ -574,6 +625,9 @@
     <t xml:space="preserve">$20–$25/hr</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aa4kgd6sbtmp</t>
+  </si>
+  <si>
     <t xml:space="preserve">Client-facing bookkeeping, like your recurring-client model</t>
   </si>
   <si>
@@ -586,6 +640,9 @@
     <t xml:space="preserve">Accounts Payable Coordinator</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aatfz6q9xtf4</t>
+  </si>
+  <si>
     <t xml:space="preserve">AP/transaction processing — core bookkeeping function</t>
   </si>
   <si>
@@ -598,6 +655,9 @@
     <t xml:space="preserve">$25.63–$31.00/hr</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aay22djqkzs4</t>
+  </si>
+  <si>
     <t xml:space="preserve">Payroll at a Manchester bookkeeping firm; you list payroll review</t>
   </si>
   <si>
@@ -613,6 +673,9 @@
     <t xml:space="preserve">From $56,000</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aaph7dxt762l</t>
+  </si>
+  <si>
     <t xml:space="preserve">AR + payroll role within commuting distance</t>
   </si>
   <si>
@@ -631,6 +694,9 @@
     <t xml:space="preserve">$44,540–$57,356</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aaqvns2cnd8q</t>
+  </si>
+  <si>
     <t xml:space="preserve">Nonprofit accounting coordination; reconciliations &amp; reporting</t>
   </si>
   <si>
@@ -652,6 +718,9 @@
     <t xml:space="preserve">$70,000–$85,000</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aagzwvczrjsl</t>
+  </si>
+  <si>
     <t xml:space="preserve">Staffing firm placement for an experienced accountant — good pay</t>
   </si>
   <si>
@@ -667,6 +736,9 @@
     <t xml:space="preserve">$94,959–$118,700</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aagnx8j42zdy</t>
+  </si>
+  <si>
     <t xml:space="preserve">Corporate accountant, strong salary; reach role with upside</t>
   </si>
   <si>
@@ -679,6 +751,9 @@
     <t xml:space="preserve">$15–$40/hr</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aakg8s2nsqlb</t>
+  </si>
+  <si>
     <t xml:space="preserve">Leverages your 200+ returns of tax-prep experience</t>
   </si>
   <si>
@@ -694,6 +769,9 @@
     <t xml:space="preserve">$27–$41/hr</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aa4k6ln4yhdj</t>
+  </si>
+  <si>
     <t xml:space="preserve">Seasonal/flexible tax prep — matches your 1040/Sch C/S-corp work</t>
   </si>
   <si>
@@ -712,6 +790,9 @@
     <t xml:space="preserve">$100,000–$150,000</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aay8bxlp2jhm</t>
+  </si>
+  <si>
     <t xml:space="preserve">Reach role for your CPA pathway (125/150 credits); top pay</t>
   </si>
   <si>
@@ -733,6 +814,9 @@
     <t xml:space="preserve">$82,779–$140,723</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aa6bykh42c27</t>
+  </si>
+  <si>
     <t xml:space="preserve">Program finance/analysis; hybrid, high ceiling</t>
   </si>
   <si>
@@ -748,6 +832,9 @@
     <t xml:space="preserve">Boston, MA</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aarswx9rsgg8</t>
+  </si>
+  <si>
     <t xml:space="preserve">Outsourced accounting — direct parallel to your fractional-CFO role</t>
   </si>
   <si>
@@ -766,6 +853,9 @@
     <t xml:space="preserve">$30–$34/hr</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aaszbvtnmqgd</t>
+  </si>
+  <si>
     <t xml:space="preserve">Hybrid staff accountant + bookkeeper; exactly your profile</t>
   </si>
   <si>
@@ -784,6 +874,9 @@
     <t xml:space="preserve">$25–$35/hr</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aazrgznjy9nf</t>
+  </si>
+  <si>
     <t xml:space="preserve">Small-business full-charge bookkeeping</t>
   </si>
   <si>
@@ -802,6 +895,9 @@
     <t xml:space="preserve">$22–$32/hr</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aar9jthdmd6m</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bookkeeping firm — multi-client QBO work like yours</t>
   </si>
   <si>
@@ -820,6 +916,9 @@
     <t xml:space="preserve">$23–$28/hr</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aahggs7qsv2t</t>
+  </si>
+  <si>
     <t xml:space="preserve">High-volume transaction reconciliation; fresh posting</t>
   </si>
   <si>
@@ -838,6 +937,9 @@
     <t xml:space="preserve">$24–$26/hr</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aabxzz7wbksg</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bookkeeping/finance support at a school</t>
   </si>
   <si>
@@ -856,6 +958,9 @@
     <t xml:space="preserve">$55,000–$75,000</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aa7bgbfgdsvq</t>
+  </si>
+  <si>
     <t xml:space="preserve">Full-cycle accounting specialist with good range</t>
   </si>
   <si>
@@ -871,6 +976,9 @@
     <t xml:space="preserve">$65,000–$75,000</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aagcmn2bgpkl</t>
+  </si>
+  <si>
     <t xml:space="preserve">Full-cycle property accounting; month-end close focus</t>
   </si>
   <si>
@@ -886,6 +994,9 @@
     <t xml:space="preserve">$77,000–$94,000</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aa6kytzgsfc9</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cost/unit-economics analysis — maps to your SKU-level work</t>
   </si>
   <si>
@@ -904,6 +1015,9 @@
     <t xml:space="preserve">From $70,000</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aa2kp46gqspf</t>
+  </si>
+  <si>
     <t xml:space="preserve">Entry CPA-firm tax role; uses your tax-prep background</t>
   </si>
   <si>
@@ -919,6 +1033,9 @@
     <t xml:space="preserve">Cambridge, MA</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aaxvy66h9pbv</t>
+  </si>
+  <si>
     <t xml:space="preserve">CPA-firm tax accountant; strong pay for your tax experience</t>
   </si>
   <si>
@@ -934,6 +1051,9 @@
     <t xml:space="preserve">$85,000–$120,000</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aajwldks9z8f</t>
+  </si>
+  <si>
     <t xml:space="preserve">Senior accountant, high pay — reach role with full-cycle duties</t>
   </si>
   <si>
@@ -952,6 +1072,9 @@
     <t xml:space="preserve">$70,600–$110,400</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aaqcrksckysy</t>
+  </si>
+  <si>
     <t xml:space="preserve">Financial analysis at a major brand; your e-commerce/retail angle</t>
   </si>
   <si>
@@ -967,6 +1090,9 @@
     <t xml:space="preserve">$105,000–$125,000</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aap2xlmscfpk</t>
+  </si>
+  <si>
     <t xml:space="preserve">Strategic FP&amp;A; variance analysis &amp; forecasting — high ceiling</t>
   </si>
   <si>
@@ -982,6 +1108,9 @@
     <t xml:space="preserve">$56,615–$76,613</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aamzf2mnbbvv</t>
+  </si>
+  <si>
     <t xml:space="preserve">Healthcare financial analysis; reconciliation-heavy</t>
   </si>
   <si>
@@ -1000,6 +1129,9 @@
     <t xml:space="preserve">$65,000–$90,000</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aarjzv4yn92x</t>
+  </si>
+  <si>
     <t xml:space="preserve">FP&amp;A / cash-flow analysis matching your reporting strengths</t>
   </si>
   <si>
@@ -1015,6 +1147,9 @@
     <t xml:space="preserve">$89,600–$134,400</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aa46td7q2glh</t>
+  </si>
+  <si>
     <t xml:space="preserve">FP&amp;A at a large employer; reach role, excellent pay</t>
   </si>
   <si>
@@ -1033,6 +1168,9 @@
     <t xml:space="preserve">$58,000–$64,000</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aa2gprnx4j7z</t>
+  </si>
+  <si>
     <t xml:space="preserve">Manufacturing staff accountant; full-cycle duties</t>
   </si>
   <si>
@@ -1051,6 +1189,9 @@
     <t xml:space="preserve">$25–$28/hr</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aa6fwcg78vsx</t>
+  </si>
+  <si>
     <t xml:space="preserve">Entry junior accountant; good foot-in-door role</t>
   </si>
   <si>
@@ -1069,6 +1210,9 @@
     <t xml:space="preserve">$75,000</t>
   </si>
   <si>
+    <t xml:space="preserve">https://to.indeed.com/aajxwjry2ssr</t>
+  </si>
+  <si>
     <t xml:space="preserve">Dealership accountant; transaction reconciliation at scale</t>
   </si>
   <si>
@@ -1082,6 +1226,9 @@
   </si>
   <si>
     <t xml:space="preserve">$83,200–$93,600</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://to.indeed.com/aa4q4nmv9jr6</t>
   </si>
   <si>
     <t xml:space="preserve">Accounting specialist with strong pay; full-cycle work</t>
@@ -1675,7 +1822,8 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="9"/>
+      <u val="single"/>
+      <sz val="8"/>
       <color rgb="FF2E75B6"/>
       <name val="Arial"/>
       <family val="0"/>
@@ -2028,7 +2176,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="20" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -2048,7 +2196,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="19" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -2618,11 +2766,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="28674714"/>
-        <c:axId val="10750514"/>
+        <c:axId val="95673138"/>
+        <c:axId val="33202770"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="28674714"/>
+        <c:axId val="95673138"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2654,7 +2802,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="10750514"/>
+        <c:crossAx val="33202770"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2662,7 +2810,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="10750514"/>
+        <c:axId val="33202770"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2704,7 +2852,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="28674714"/>
+        <c:crossAx val="95673138"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3031,11 +3179,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="18801675"/>
-        <c:axId val="56911843"/>
+        <c:axId val="66263137"/>
+        <c:axId val="2691430"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="18801675"/>
+        <c:axId val="66263137"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3067,7 +3215,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="56911843"/>
+        <c:crossAx val="2691430"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3075,7 +3223,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="56911843"/>
+        <c:axId val="2691430"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3107,7 +3255,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="18801675"/>
+        <c:crossAx val="66263137"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3379,11 +3527,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="56763706"/>
-        <c:axId val="98752451"/>
+        <c:axId val="71698190"/>
+        <c:axId val="2111968"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="56763706"/>
+        <c:axId val="71698190"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3415,7 +3563,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="98752451"/>
+        <c:crossAx val="2111968"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3423,7 +3571,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="98752451"/>
+        <c:axId val="2111968"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3455,7 +3603,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="56763706"/>
+        <c:crossAx val="71698190"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3734,11 +3882,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="55440154"/>
-        <c:axId val="94490151"/>
+        <c:axId val="32428152"/>
+        <c:axId val="56366579"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="55440154"/>
+        <c:axId val="32428152"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3770,7 +3918,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94490151"/>
+        <c:crossAx val="56366579"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3778,7 +3926,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="94490151"/>
+        <c:axId val="56366579"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3810,7 +3958,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="55440154"/>
+        <c:crossAx val="32428152"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4281,7 +4429,7 @@
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="str">
         <f aca="true">"Updated:  "&amp;TEXT(TODAY(),"dddd, mmm d, yyyy")&amp;"   (times in Eastern)"</f>
-        <v>Updated:  Friday, Oct 23, 2026   (times in Eastern)</v>
+        <v>Updated:  Sunday, Oct 25, 2026   (times in Eastern)</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
@@ -4971,7 +5119,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="11" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="15"/>
@@ -5221,13 +5369,13 @@
         <v>43</v>
       </c>
       <c r="O3" s="45" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="P3" s="41" t="n">
         <v>5</v>
       </c>
       <c r="Q3" s="43" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="R3" s="41" t="s">
         <v>85</v>
@@ -5267,7 +5415,7 @@
     </row>
     <row r="4" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="36" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B4" s="37" t="n">
         <v>46318</v>
@@ -5279,13 +5427,13 @@
         <v>35</v>
       </c>
       <c r="E4" s="36" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F4" s="38" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G4" s="36" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H4" s="36" t="s">
         <v>80</v>
@@ -5294,7 +5442,7 @@
         <v>89</v>
       </c>
       <c r="J4" s="36" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K4" s="39" t="n">
         <v>65000</v>
@@ -5310,13 +5458,13 @@
         <v>43</v>
       </c>
       <c r="O4" s="40" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="P4" s="36" t="n">
         <v>5</v>
       </c>
       <c r="Q4" s="38" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="R4" s="36" t="s">
         <v>85</v>
@@ -5356,7 +5504,7 @@
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="41" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B5" s="42" t="n">
         <v>46318</v>
@@ -5368,13 +5516,13 @@
         <v>35</v>
       </c>
       <c r="E5" s="41" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F5" s="43" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G5" s="41" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H5" s="41" t="s">
         <v>80</v>
@@ -5383,7 +5531,7 @@
         <v>89</v>
       </c>
       <c r="J5" s="41" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="K5" s="44" t="n">
         <v>58380</v>
@@ -5399,13 +5547,13 @@
         <v>43</v>
       </c>
       <c r="O5" s="45" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="P5" s="41" t="n">
         <v>5</v>
       </c>
       <c r="Q5" s="43" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="R5" s="41" t="s">
         <v>85</v>
@@ -5445,7 +5593,7 @@
     </row>
     <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="36" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B6" s="37" t="n">
         <v>46318</v>
@@ -5457,13 +5605,13 @@
         <v>31</v>
       </c>
       <c r="E6" s="36" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="F6" s="38" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="G6" s="36" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H6" s="36" t="s">
         <v>80</v>
@@ -5472,7 +5620,7 @@
         <v>89</v>
       </c>
       <c r="J6" s="36" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="K6" s="39" t="n">
         <v>62400</v>
@@ -5488,13 +5636,13 @@
         <v>43</v>
       </c>
       <c r="O6" s="40" t="s">
-        <v>83</v>
+        <v>109</v>
       </c>
       <c r="P6" s="36" t="n">
         <v>5</v>
       </c>
       <c r="Q6" s="38" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="R6" s="36" t="s">
         <v>85</v>
@@ -5534,7 +5682,7 @@
     </row>
     <row r="7" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="41" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B7" s="42" t="n">
         <v>46318</v>
@@ -5546,13 +5694,13 @@
         <v>31</v>
       </c>
       <c r="E7" s="41" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="F7" s="43" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="G7" s="41" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H7" s="41" t="s">
         <v>80</v>
@@ -5561,7 +5709,7 @@
         <v>89</v>
       </c>
       <c r="J7" s="41" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="K7" s="44" t="n">
         <v>50000</v>
@@ -5577,13 +5725,13 @@
         <v>43</v>
       </c>
       <c r="O7" s="45" t="s">
-        <v>83</v>
+        <v>115</v>
       </c>
       <c r="P7" s="41" t="n">
         <v>3</v>
       </c>
       <c r="Q7" s="43" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="R7" s="41" t="s">
         <v>85</v>
@@ -5623,7 +5771,7 @@
     </row>
     <row r="8" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="36" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="B8" s="37" t="n">
         <v>46318</v>
@@ -5635,13 +5783,13 @@
         <v>31</v>
       </c>
       <c r="E8" s="36" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="F8" s="38" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G8" s="36" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="H8" s="36" t="s">
         <v>80</v>
@@ -5650,7 +5798,7 @@
         <v>89</v>
       </c>
       <c r="J8" s="36" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="K8" s="39" t="n">
         <v>62000</v>
@@ -5666,13 +5814,13 @@
         <v>43</v>
       </c>
       <c r="O8" s="40" t="s">
-        <v>83</v>
+        <v>122</v>
       </c>
       <c r="P8" s="36" t="n">
         <v>5</v>
       </c>
       <c r="Q8" s="38" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="R8" s="36" t="s">
         <v>85</v>
@@ -5712,7 +5860,7 @@
     </row>
     <row r="9" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="41" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="B9" s="42" t="n">
         <v>46318</v>
@@ -5724,13 +5872,13 @@
         <v>31</v>
       </c>
       <c r="E9" s="41" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="F9" s="43" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="G9" s="41" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="H9" s="41" t="s">
         <v>80</v>
@@ -5739,7 +5887,7 @@
         <v>89</v>
       </c>
       <c r="J9" s="41" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="K9" s="44" t="n">
         <v>41600</v>
@@ -5755,13 +5903,13 @@
         <v>43</v>
       </c>
       <c r="O9" s="45" t="s">
-        <v>83</v>
+        <v>129</v>
       </c>
       <c r="P9" s="41" t="n">
         <v>3</v>
       </c>
       <c r="Q9" s="43" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="R9" s="41" t="s">
         <v>85</v>
@@ -5801,7 +5949,7 @@
     </row>
     <row r="10" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="36" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="B10" s="37" t="n">
         <v>46318</v>
@@ -5813,13 +5961,13 @@
         <v>29</v>
       </c>
       <c r="E10" s="36" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="F10" s="38" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="G10" s="36" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="H10" s="36" t="s">
         <v>80</v>
@@ -5828,7 +5976,7 @@
         <v>89</v>
       </c>
       <c r="J10" s="36" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="K10" s="39" t="n">
         <v>58000</v>
@@ -5844,13 +5992,13 @@
         <v>43</v>
       </c>
       <c r="O10" s="40" t="s">
-        <v>83</v>
+        <v>136</v>
       </c>
       <c r="P10" s="36" t="n">
         <v>5</v>
       </c>
       <c r="Q10" s="38" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="R10" s="36" t="s">
         <v>85</v>
@@ -5890,7 +6038,7 @@
     </row>
     <row r="11" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="41" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="B11" s="42" t="n">
         <v>46318</v>
@@ -5902,13 +6050,13 @@
         <v>31</v>
       </c>
       <c r="E11" s="41" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="F11" s="43" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="G11" s="41" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="H11" s="41" t="s">
         <v>80</v>
@@ -5917,7 +6065,7 @@
         <v>89</v>
       </c>
       <c r="J11" s="41" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="K11" s="44" t="n">
         <v>54930</v>
@@ -5933,13 +6081,13 @@
         <v>43</v>
       </c>
       <c r="O11" s="45" t="s">
-        <v>83</v>
+        <v>143</v>
       </c>
       <c r="P11" s="41" t="n">
         <v>5</v>
       </c>
       <c r="Q11" s="43" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="R11" s="41" t="s">
         <v>85</v>
@@ -5979,7 +6127,7 @@
     </row>
     <row r="12" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="36" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="B12" s="37" t="n">
         <v>46318</v>
@@ -5991,13 +6139,13 @@
         <v>31</v>
       </c>
       <c r="E12" s="36" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="F12" s="38" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="G12" s="36" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="H12" s="36" t="s">
         <v>80</v>
@@ -6006,7 +6154,7 @@
         <v>89</v>
       </c>
       <c r="J12" s="36" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="K12" s="39"/>
       <c r="L12" s="39"/>
@@ -6018,13 +6166,13 @@
         <v>43</v>
       </c>
       <c r="O12" s="40" t="s">
-        <v>83</v>
+        <v>150</v>
       </c>
       <c r="P12" s="36" t="n">
         <v>3</v>
       </c>
       <c r="Q12" s="38" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
       <c r="R12" s="36" t="s">
         <v>85</v>
@@ -6064,7 +6212,7 @@
     </row>
     <row r="13" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="41" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="B13" s="42" t="n">
         <v>46318</v>
@@ -6076,13 +6224,13 @@
         <v>33</v>
       </c>
       <c r="E13" s="41" t="s">
-        <v>143</v>
+        <v>153</v>
       </c>
       <c r="F13" s="43" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
       <c r="G13" s="41" t="s">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="H13" s="41" t="s">
         <v>80</v>
@@ -6091,7 +6239,7 @@
         <v>89</v>
       </c>
       <c r="J13" s="41" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="K13" s="44" t="n">
         <v>60000</v>
@@ -6107,13 +6255,13 @@
         <v>43</v>
       </c>
       <c r="O13" s="45" t="s">
-        <v>83</v>
+        <v>157</v>
       </c>
       <c r="P13" s="41" t="n">
         <v>5</v>
       </c>
       <c r="Q13" s="43" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="R13" s="41" t="s">
         <v>85</v>
@@ -6153,7 +6301,7 @@
     </row>
     <row r="14" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="36" t="s">
-        <v>148</v>
+        <v>159</v>
       </c>
       <c r="B14" s="37" t="n">
         <v>46318</v>
@@ -6165,10 +6313,10 @@
         <v>31</v>
       </c>
       <c r="E14" s="36" t="s">
-        <v>149</v>
+        <v>160</v>
       </c>
       <c r="F14" s="38" t="s">
-        <v>150</v>
+        <v>161</v>
       </c>
       <c r="G14" s="36" t="s">
         <v>79</v>
@@ -6180,7 +6328,7 @@
         <v>89</v>
       </c>
       <c r="J14" s="36" t="s">
-        <v>151</v>
+        <v>162</v>
       </c>
       <c r="K14" s="39" t="n">
         <v>45760</v>
@@ -6196,13 +6344,13 @@
         <v>43</v>
       </c>
       <c r="O14" s="40" t="s">
-        <v>83</v>
+        <v>163</v>
       </c>
       <c r="P14" s="36" t="n">
         <v>5</v>
       </c>
       <c r="Q14" s="38" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="R14" s="36" t="s">
         <v>85</v>
@@ -6242,7 +6390,7 @@
     </row>
     <row r="15" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="41" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="B15" s="42" t="n">
         <v>46318</v>
@@ -6254,10 +6402,10 @@
         <v>34</v>
       </c>
       <c r="E15" s="41" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="F15" s="43" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="G15" s="41" t="s">
         <v>79</v>
@@ -6269,7 +6417,7 @@
         <v>89</v>
       </c>
       <c r="J15" s="41" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="K15" s="44" t="n">
         <v>75000</v>
@@ -6285,13 +6433,13 @@
         <v>43</v>
       </c>
       <c r="O15" s="45" t="s">
-        <v>83</v>
+        <v>169</v>
       </c>
       <c r="P15" s="41" t="n">
         <v>5</v>
       </c>
       <c r="Q15" s="43" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="R15" s="41" t="s">
         <v>85</v>
@@ -6331,7 +6479,7 @@
     </row>
     <row r="16" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="36" t="s">
-        <v>158</v>
+        <v>171</v>
       </c>
       <c r="B16" s="37" t="n">
         <v>46318</v>
@@ -6343,10 +6491,10 @@
         <v>33</v>
       </c>
       <c r="E16" s="36" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="F16" s="38" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="G16" s="36" t="s">
         <v>79</v>
@@ -6358,7 +6506,7 @@
         <v>81</v>
       </c>
       <c r="J16" s="36" t="s">
-        <v>161</v>
+        <v>174</v>
       </c>
       <c r="K16" s="39" t="n">
         <v>83200</v>
@@ -6372,13 +6520,13 @@
         <v>43</v>
       </c>
       <c r="O16" s="40" t="s">
-        <v>83</v>
+        <v>175</v>
       </c>
       <c r="P16" s="36" t="n">
         <v>3</v>
       </c>
       <c r="Q16" s="38" t="s">
-        <v>162</v>
+        <v>176</v>
       </c>
       <c r="R16" s="36" t="s">
         <v>85</v>
@@ -6418,7 +6566,7 @@
     </row>
     <row r="17" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="41" t="s">
-        <v>163</v>
+        <v>177</v>
       </c>
       <c r="B17" s="42" t="n">
         <v>46318</v>
@@ -6430,13 +6578,13 @@
         <v>32</v>
       </c>
       <c r="E17" s="41" t="s">
-        <v>164</v>
+        <v>178</v>
       </c>
       <c r="F17" s="43" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="G17" s="41" t="s">
-        <v>166</v>
+        <v>180</v>
       </c>
       <c r="H17" s="41" t="s">
         <v>80</v>
@@ -6445,7 +6593,7 @@
         <v>89</v>
       </c>
       <c r="J17" s="41" t="s">
-        <v>167</v>
+        <v>181</v>
       </c>
       <c r="K17" s="44" t="n">
         <v>60424</v>
@@ -6461,13 +6609,13 @@
         <v>43</v>
       </c>
       <c r="O17" s="45" t="s">
-        <v>83</v>
+        <v>182</v>
       </c>
       <c r="P17" s="41" t="n">
         <v>3</v>
       </c>
       <c r="Q17" s="43" t="s">
-        <v>168</v>
+        <v>183</v>
       </c>
       <c r="R17" s="41" t="s">
         <v>85</v>
@@ -6507,7 +6655,7 @@
     </row>
     <row r="18" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="36" t="s">
-        <v>169</v>
+        <v>184</v>
       </c>
       <c r="B18" s="37" t="n">
         <v>46318</v>
@@ -6519,13 +6667,13 @@
         <v>32</v>
       </c>
       <c r="E18" s="36" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F18" s="38" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
       <c r="G18" s="36" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="H18" s="36" t="s">
         <v>80</v>
@@ -6534,7 +6682,7 @@
         <v>89</v>
       </c>
       <c r="J18" s="36" t="s">
-        <v>172</v>
+        <v>187</v>
       </c>
       <c r="K18" s="39" t="n">
         <v>64000</v>
@@ -6550,13 +6698,13 @@
         <v>43</v>
       </c>
       <c r="O18" s="40" t="s">
-        <v>83</v>
+        <v>188</v>
       </c>
       <c r="P18" s="36" t="n">
         <v>3</v>
       </c>
       <c r="Q18" s="38" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
       <c r="R18" s="36" t="s">
         <v>85</v>
@@ -6596,7 +6744,7 @@
     </row>
     <row r="19" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="41" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
       <c r="B19" s="42" t="n">
         <v>46318</v>
@@ -6608,13 +6756,13 @@
         <v>31</v>
       </c>
       <c r="E19" s="41" t="s">
-        <v>175</v>
+        <v>191</v>
       </c>
       <c r="F19" s="43" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="G19" s="41" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="H19" s="41" t="s">
         <v>80</v>
@@ -6623,7 +6771,7 @@
         <v>89</v>
       </c>
       <c r="J19" s="41" t="s">
-        <v>177</v>
+        <v>193</v>
       </c>
       <c r="K19" s="44" t="n">
         <v>80000</v>
@@ -6639,13 +6787,13 @@
         <v>43</v>
       </c>
       <c r="O19" s="45" t="s">
-        <v>83</v>
+        <v>194</v>
       </c>
       <c r="P19" s="41" t="n">
         <v>3</v>
       </c>
       <c r="Q19" s="43" t="s">
-        <v>178</v>
+        <v>195</v>
       </c>
       <c r="R19" s="41" t="s">
         <v>85</v>
@@ -6685,7 +6833,7 @@
     </row>
     <row r="20" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="36" t="s">
-        <v>179</v>
+        <v>196</v>
       </c>
       <c r="B20" s="37" t="n">
         <v>46318</v>
@@ -6697,13 +6845,13 @@
         <v>31</v>
       </c>
       <c r="E20" s="36" t="s">
-        <v>175</v>
+        <v>191</v>
       </c>
       <c r="F20" s="38" t="s">
-        <v>180</v>
+        <v>197</v>
       </c>
       <c r="G20" s="36" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="H20" s="36" t="s">
         <v>80</v>
@@ -6712,7 +6860,7 @@
         <v>89</v>
       </c>
       <c r="J20" s="36" t="s">
-        <v>181</v>
+        <v>198</v>
       </c>
       <c r="K20" s="39" t="n">
         <v>41600</v>
@@ -6728,13 +6876,13 @@
         <v>43</v>
       </c>
       <c r="O20" s="40" t="s">
-        <v>83</v>
+        <v>199</v>
       </c>
       <c r="P20" s="36" t="n">
         <v>5</v>
       </c>
       <c r="Q20" s="38" t="s">
-        <v>182</v>
+        <v>200</v>
       </c>
       <c r="R20" s="36" t="s">
         <v>85</v>
@@ -6774,7 +6922,7 @@
     </row>
     <row r="21" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="41" t="s">
-        <v>183</v>
+        <v>201</v>
       </c>
       <c r="B21" s="42" t="n">
         <v>46318</v>
@@ -6786,22 +6934,22 @@
         <v>31</v>
       </c>
       <c r="E21" s="41" t="s">
-        <v>184</v>
+        <v>202</v>
       </c>
       <c r="F21" s="43" t="s">
-        <v>185</v>
+        <v>203</v>
       </c>
       <c r="G21" s="41" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="H21" s="41" t="s">
         <v>80</v>
       </c>
       <c r="I21" s="41" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="J21" s="41" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="K21" s="44"/>
       <c r="L21" s="44"/>
@@ -6813,13 +6961,13 @@
         <v>43</v>
       </c>
       <c r="O21" s="45" t="s">
-        <v>83</v>
+        <v>204</v>
       </c>
       <c r="P21" s="41" t="n">
         <v>3</v>
       </c>
       <c r="Q21" s="43" t="s">
-        <v>186</v>
+        <v>205</v>
       </c>
       <c r="R21" s="41" t="s">
         <v>85</v>
@@ -6859,7 +7007,7 @@
     </row>
     <row r="22" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="36" t="s">
-        <v>187</v>
+        <v>206</v>
       </c>
       <c r="B22" s="37" t="n">
         <v>46318</v>
@@ -6874,7 +7022,7 @@
         <v>87</v>
       </c>
       <c r="F22" s="38" t="s">
-        <v>188</v>
+        <v>207</v>
       </c>
       <c r="G22" s="36" t="s">
         <v>79</v>
@@ -6886,7 +7034,7 @@
         <v>89</v>
       </c>
       <c r="J22" s="36" t="s">
-        <v>189</v>
+        <v>208</v>
       </c>
       <c r="K22" s="39" t="n">
         <v>53310</v>
@@ -6902,13 +7050,13 @@
         <v>43</v>
       </c>
       <c r="O22" s="40" t="s">
-        <v>83</v>
+        <v>209</v>
       </c>
       <c r="P22" s="36" t="n">
         <v>3</v>
       </c>
       <c r="Q22" s="38" t="s">
-        <v>190</v>
+        <v>210</v>
       </c>
       <c r="R22" s="36" t="s">
         <v>85</v>
@@ -6948,7 +7096,7 @@
     </row>
     <row r="23" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="41" t="s">
-        <v>191</v>
+        <v>211</v>
       </c>
       <c r="B23" s="42" t="n">
         <v>46318</v>
@@ -6960,13 +7108,13 @@
         <v>31</v>
       </c>
       <c r="E23" s="41" t="s">
-        <v>192</v>
+        <v>212</v>
       </c>
       <c r="F23" s="43" t="s">
-        <v>193</v>
+        <v>213</v>
       </c>
       <c r="G23" s="41" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="H23" s="41" t="s">
         <v>80</v>
@@ -6975,7 +7123,7 @@
         <v>89</v>
       </c>
       <c r="J23" s="41" t="s">
-        <v>194</v>
+        <v>214</v>
       </c>
       <c r="K23" s="44" t="n">
         <v>56000</v>
@@ -6989,13 +7137,13 @@
         <v>43</v>
       </c>
       <c r="O23" s="45" t="s">
-        <v>83</v>
+        <v>215</v>
       </c>
       <c r="P23" s="41" t="n">
         <v>3</v>
       </c>
       <c r="Q23" s="43" t="s">
-        <v>195</v>
+        <v>216</v>
       </c>
       <c r="R23" s="41" t="s">
         <v>85</v>
@@ -7035,7 +7183,7 @@
     </row>
     <row r="24" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="36" t="s">
-        <v>196</v>
+        <v>217</v>
       </c>
       <c r="B24" s="37" t="n">
         <v>46318</v>
@@ -7047,13 +7195,13 @@
         <v>33</v>
       </c>
       <c r="E24" s="36" t="s">
-        <v>197</v>
+        <v>218</v>
       </c>
       <c r="F24" s="38" t="s">
-        <v>198</v>
+        <v>219</v>
       </c>
       <c r="G24" s="36" t="s">
-        <v>199</v>
+        <v>220</v>
       </c>
       <c r="H24" s="36" t="s">
         <v>80</v>
@@ -7062,7 +7210,7 @@
         <v>89</v>
       </c>
       <c r="J24" s="36" t="s">
-        <v>200</v>
+        <v>221</v>
       </c>
       <c r="K24" s="39" t="n">
         <v>44540</v>
@@ -7078,13 +7226,13 @@
         <v>43</v>
       </c>
       <c r="O24" s="40" t="s">
-        <v>83</v>
+        <v>222</v>
       </c>
       <c r="P24" s="36" t="n">
         <v>3</v>
       </c>
       <c r="Q24" s="38" t="s">
-        <v>201</v>
+        <v>223</v>
       </c>
       <c r="R24" s="36" t="s">
         <v>85</v>
@@ -7124,7 +7272,7 @@
     </row>
     <row r="25" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="41" t="s">
-        <v>202</v>
+        <v>224</v>
       </c>
       <c r="B25" s="42" t="n">
         <v>46318</v>
@@ -7136,22 +7284,22 @@
         <v>31</v>
       </c>
       <c r="E25" s="41" t="s">
-        <v>203</v>
+        <v>225</v>
       </c>
       <c r="F25" s="43" t="s">
-        <v>204</v>
+        <v>226</v>
       </c>
       <c r="G25" s="41" t="s">
-        <v>205</v>
+        <v>227</v>
       </c>
       <c r="H25" s="41" t="s">
         <v>80</v>
       </c>
       <c r="I25" s="41" t="s">
-        <v>206</v>
+        <v>228</v>
       </c>
       <c r="J25" s="41" t="s">
-        <v>207</v>
+        <v>229</v>
       </c>
       <c r="K25" s="44" t="n">
         <v>70000</v>
@@ -7167,13 +7315,13 @@
         <v>43</v>
       </c>
       <c r="O25" s="45" t="s">
-        <v>83</v>
+        <v>230</v>
       </c>
       <c r="P25" s="41" t="n">
         <v>5</v>
       </c>
       <c r="Q25" s="43" t="s">
-        <v>208</v>
+        <v>231</v>
       </c>
       <c r="R25" s="41" t="s">
         <v>85</v>
@@ -7213,7 +7361,7 @@
     </row>
     <row r="26" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="36" t="s">
-        <v>209</v>
+        <v>232</v>
       </c>
       <c r="B26" s="37" t="n">
         <v>46318</v>
@@ -7225,13 +7373,13 @@
         <v>34</v>
       </c>
       <c r="E26" s="36" t="s">
-        <v>210</v>
+        <v>233</v>
       </c>
       <c r="F26" s="38" t="s">
-        <v>211</v>
+        <v>234</v>
       </c>
       <c r="G26" s="36" t="s">
-        <v>205</v>
+        <v>227</v>
       </c>
       <c r="H26" s="36" t="s">
         <v>80</v>
@@ -7240,7 +7388,7 @@
         <v>89</v>
       </c>
       <c r="J26" s="36" t="s">
-        <v>212</v>
+        <v>235</v>
       </c>
       <c r="K26" s="39" t="n">
         <v>94959</v>
@@ -7256,13 +7404,13 @@
         <v>43</v>
       </c>
       <c r="O26" s="40" t="s">
-        <v>83</v>
+        <v>236</v>
       </c>
       <c r="P26" s="36" t="n">
         <v>3</v>
       </c>
       <c r="Q26" s="38" t="s">
-        <v>213</v>
+        <v>237</v>
       </c>
       <c r="R26" s="36" t="s">
         <v>85</v>
@@ -7302,7 +7450,7 @@
     </row>
     <row r="27" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="41" t="s">
-        <v>214</v>
+        <v>238</v>
       </c>
       <c r="B27" s="42" t="n">
         <v>46318</v>
@@ -7317,7 +7465,7 @@
         <v>77</v>
       </c>
       <c r="F27" s="43" t="s">
-        <v>215</v>
+        <v>239</v>
       </c>
       <c r="G27" s="41" t="s">
         <v>79</v>
@@ -7329,7 +7477,7 @@
         <v>81</v>
       </c>
       <c r="J27" s="41" t="s">
-        <v>216</v>
+        <v>240</v>
       </c>
       <c r="K27" s="44" t="n">
         <v>31200</v>
@@ -7345,13 +7493,13 @@
         <v>43</v>
       </c>
       <c r="O27" s="45" t="s">
-        <v>83</v>
+        <v>241</v>
       </c>
       <c r="P27" s="41" t="n">
         <v>3</v>
       </c>
       <c r="Q27" s="43" t="s">
-        <v>217</v>
+        <v>242</v>
       </c>
       <c r="R27" s="41" t="s">
         <v>85</v>
@@ -7391,7 +7539,7 @@
     </row>
     <row r="28" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="36" t="s">
-        <v>218</v>
+        <v>243</v>
       </c>
       <c r="B28" s="37" t="n">
         <v>46318</v>
@@ -7403,22 +7551,22 @@
         <v>36</v>
       </c>
       <c r="E28" s="36" t="s">
-        <v>219</v>
+        <v>244</v>
       </c>
       <c r="F28" s="38" t="s">
-        <v>220</v>
+        <v>245</v>
       </c>
       <c r="G28" s="36" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="H28" s="36" t="s">
         <v>80</v>
       </c>
       <c r="I28" s="36" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="J28" s="36" t="s">
-        <v>221</v>
+        <v>246</v>
       </c>
       <c r="K28" s="39" t="n">
         <v>56160</v>
@@ -7434,13 +7582,13 @@
         <v>43</v>
       </c>
       <c r="O28" s="40" t="s">
-        <v>83</v>
+        <v>247</v>
       </c>
       <c r="P28" s="36" t="n">
         <v>3</v>
       </c>
       <c r="Q28" s="38" t="s">
-        <v>222</v>
+        <v>248</v>
       </c>
       <c r="R28" s="36" t="s">
         <v>85</v>
@@ -7480,7 +7628,7 @@
     </row>
     <row r="29" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="41" t="s">
-        <v>223</v>
+        <v>249</v>
       </c>
       <c r="B29" s="42" t="n">
         <v>46318</v>
@@ -7492,13 +7640,13 @@
         <v>31</v>
       </c>
       <c r="E29" s="41" t="s">
-        <v>224</v>
+        <v>250</v>
       </c>
       <c r="F29" s="43" t="s">
-        <v>225</v>
+        <v>251</v>
       </c>
       <c r="G29" s="41" t="s">
-        <v>226</v>
+        <v>252</v>
       </c>
       <c r="H29" s="41" t="s">
         <v>80</v>
@@ -7507,7 +7655,7 @@
         <v>89</v>
       </c>
       <c r="J29" s="41" t="s">
-        <v>227</v>
+        <v>253</v>
       </c>
       <c r="K29" s="44" t="n">
         <v>100000</v>
@@ -7523,13 +7671,13 @@
         <v>43</v>
       </c>
       <c r="O29" s="45" t="s">
-        <v>83</v>
+        <v>254</v>
       </c>
       <c r="P29" s="41" t="n">
         <v>3</v>
       </c>
       <c r="Q29" s="43" t="s">
-        <v>228</v>
+        <v>255</v>
       </c>
       <c r="R29" s="41" t="s">
         <v>85</v>
@@ -7569,7 +7717,7 @@
     </row>
     <row r="30" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="36" t="s">
-        <v>229</v>
+        <v>256</v>
       </c>
       <c r="B30" s="37" t="n">
         <v>46318</v>
@@ -7581,22 +7729,22 @@
         <v>34</v>
       </c>
       <c r="E30" s="36" t="s">
-        <v>230</v>
+        <v>257</v>
       </c>
       <c r="F30" s="38" t="s">
-        <v>231</v>
+        <v>258</v>
       </c>
       <c r="G30" s="36" t="s">
-        <v>232</v>
+        <v>259</v>
       </c>
       <c r="H30" s="36" t="s">
-        <v>233</v>
+        <v>260</v>
       </c>
       <c r="I30" s="36" t="s">
         <v>89</v>
       </c>
       <c r="J30" s="36" t="s">
-        <v>234</v>
+        <v>261</v>
       </c>
       <c r="K30" s="39" t="n">
         <v>82779</v>
@@ -7612,13 +7760,13 @@
         <v>43</v>
       </c>
       <c r="O30" s="40" t="s">
-        <v>83</v>
+        <v>262</v>
       </c>
       <c r="P30" s="36" t="n">
         <v>3</v>
       </c>
       <c r="Q30" s="38" t="s">
-        <v>235</v>
+        <v>263</v>
       </c>
       <c r="R30" s="36" t="s">
         <v>85</v>
@@ -7658,7 +7806,7 @@
     </row>
     <row r="31" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="41" t="s">
-        <v>236</v>
+        <v>264</v>
       </c>
       <c r="B31" s="42" t="n">
         <v>46318</v>
@@ -7670,13 +7818,13 @@
         <v>29</v>
       </c>
       <c r="E31" s="41" t="s">
-        <v>237</v>
+        <v>265</v>
       </c>
       <c r="F31" s="43" t="s">
-        <v>238</v>
+        <v>266</v>
       </c>
       <c r="G31" s="41" t="s">
-        <v>239</v>
+        <v>267</v>
       </c>
       <c r="H31" s="41" t="s">
         <v>80</v>
@@ -7685,7 +7833,7 @@
         <v>81</v>
       </c>
       <c r="J31" s="41" t="s">
-        <v>207</v>
+        <v>229</v>
       </c>
       <c r="K31" s="44" t="n">
         <v>70000</v>
@@ -7701,13 +7849,13 @@
         <v>43</v>
       </c>
       <c r="O31" s="45" t="s">
-        <v>83</v>
+        <v>268</v>
       </c>
       <c r="P31" s="41" t="n">
         <v>5</v>
       </c>
       <c r="Q31" s="43" t="s">
-        <v>240</v>
+        <v>269</v>
       </c>
       <c r="R31" s="41" t="s">
         <v>85</v>
@@ -7747,7 +7895,7 @@
     </row>
     <row r="32" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="36" t="s">
-        <v>241</v>
+        <v>270</v>
       </c>
       <c r="B32" s="37" t="n">
         <v>46318</v>
@@ -7759,13 +7907,13 @@
         <v>29</v>
       </c>
       <c r="E32" s="36" t="s">
-        <v>242</v>
+        <v>271</v>
       </c>
       <c r="F32" s="38" t="s">
-        <v>243</v>
+        <v>272</v>
       </c>
       <c r="G32" s="36" t="s">
-        <v>244</v>
+        <v>273</v>
       </c>
       <c r="H32" s="36" t="s">
         <v>80</v>
@@ -7774,7 +7922,7 @@
         <v>89</v>
       </c>
       <c r="J32" s="36" t="s">
-        <v>245</v>
+        <v>274</v>
       </c>
       <c r="K32" s="39" t="n">
         <v>62400</v>
@@ -7790,13 +7938,13 @@
         <v>43</v>
       </c>
       <c r="O32" s="40" t="s">
-        <v>83</v>
+        <v>275</v>
       </c>
       <c r="P32" s="36" t="n">
         <v>5</v>
       </c>
       <c r="Q32" s="38" t="s">
-        <v>246</v>
+        <v>276</v>
       </c>
       <c r="R32" s="36" t="s">
         <v>85</v>
@@ -7836,7 +7984,7 @@
     </row>
     <row r="33" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="41" t="s">
-        <v>247</v>
+        <v>277</v>
       </c>
       <c r="B33" s="42" t="n">
         <v>46318</v>
@@ -7848,13 +7996,13 @@
         <v>31</v>
       </c>
       <c r="E33" s="41" t="s">
-        <v>248</v>
+        <v>278</v>
       </c>
       <c r="F33" s="43" t="s">
-        <v>249</v>
+        <v>279</v>
       </c>
       <c r="G33" s="41" t="s">
-        <v>250</v>
+        <v>280</v>
       </c>
       <c r="H33" s="41" t="s">
         <v>80</v>
@@ -7863,7 +8011,7 @@
         <v>81</v>
       </c>
       <c r="J33" s="41" t="s">
-        <v>251</v>
+        <v>281</v>
       </c>
       <c r="K33" s="44" t="n">
         <v>52000</v>
@@ -7879,13 +8027,13 @@
         <v>43</v>
       </c>
       <c r="O33" s="45" t="s">
-        <v>83</v>
+        <v>282</v>
       </c>
       <c r="P33" s="41" t="n">
         <v>5</v>
       </c>
       <c r="Q33" s="43" t="s">
-        <v>252</v>
+        <v>283</v>
       </c>
       <c r="R33" s="41" t="s">
         <v>85</v>
@@ -7925,7 +8073,7 @@
     </row>
     <row r="34" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="36" t="s">
-        <v>253</v>
+        <v>284</v>
       </c>
       <c r="B34" s="37" t="n">
         <v>46318</v>
@@ -7937,13 +8085,13 @@
         <v>29</v>
       </c>
       <c r="E34" s="36" t="s">
-        <v>254</v>
+        <v>285</v>
       </c>
       <c r="F34" s="38" t="s">
-        <v>255</v>
+        <v>286</v>
       </c>
       <c r="G34" s="36" t="s">
-        <v>256</v>
+        <v>287</v>
       </c>
       <c r="H34" s="36" t="s">
         <v>80</v>
@@ -7952,7 +8100,7 @@
         <v>81</v>
       </c>
       <c r="J34" s="36" t="s">
-        <v>257</v>
+        <v>288</v>
       </c>
       <c r="K34" s="39" t="n">
         <v>45760</v>
@@ -7968,13 +8116,13 @@
         <v>43</v>
       </c>
       <c r="O34" s="40" t="s">
-        <v>83</v>
+        <v>289</v>
       </c>
       <c r="P34" s="36" t="n">
         <v>5</v>
       </c>
       <c r="Q34" s="38" t="s">
-        <v>258</v>
+        <v>290</v>
       </c>
       <c r="R34" s="36" t="s">
         <v>85</v>
@@ -8014,7 +8162,7 @@
     </row>
     <row r="35" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="41" t="s">
-        <v>259</v>
+        <v>291</v>
       </c>
       <c r="B35" s="42" t="n">
         <v>46318</v>
@@ -8026,13 +8174,13 @@
         <v>31</v>
       </c>
       <c r="E35" s="41" t="s">
-        <v>260</v>
+        <v>292</v>
       </c>
       <c r="F35" s="43" t="s">
-        <v>261</v>
+        <v>293</v>
       </c>
       <c r="G35" s="41" t="s">
-        <v>262</v>
+        <v>294</v>
       </c>
       <c r="H35" s="41" t="s">
         <v>80</v>
@@ -8041,7 +8189,7 @@
         <v>89</v>
       </c>
       <c r="J35" s="41" t="s">
-        <v>263</v>
+        <v>295</v>
       </c>
       <c r="K35" s="44" t="n">
         <v>47840</v>
@@ -8057,13 +8205,13 @@
         <v>43</v>
       </c>
       <c r="O35" s="45" t="s">
-        <v>83</v>
+        <v>296</v>
       </c>
       <c r="P35" s="41" t="n">
         <v>3</v>
       </c>
       <c r="Q35" s="43" t="s">
-        <v>264</v>
+        <v>297</v>
       </c>
       <c r="R35" s="41" t="s">
         <v>85</v>
@@ -8103,7 +8251,7 @@
     </row>
     <row r="36" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="36" t="s">
-        <v>265</v>
+        <v>298</v>
       </c>
       <c r="B36" s="37" t="n">
         <v>46318</v>
@@ -8115,13 +8263,13 @@
         <v>33</v>
       </c>
       <c r="E36" s="36" t="s">
-        <v>266</v>
+        <v>299</v>
       </c>
       <c r="F36" s="38" t="s">
-        <v>267</v>
+        <v>300</v>
       </c>
       <c r="G36" s="36" t="s">
-        <v>268</v>
+        <v>301</v>
       </c>
       <c r="H36" s="36" t="s">
         <v>80</v>
@@ -8130,7 +8278,7 @@
         <v>81</v>
       </c>
       <c r="J36" s="36" t="s">
-        <v>269</v>
+        <v>302</v>
       </c>
       <c r="K36" s="39" t="n">
         <v>49920</v>
@@ -8146,13 +8294,13 @@
         <v>43</v>
       </c>
       <c r="O36" s="40" t="s">
-        <v>83</v>
+        <v>303</v>
       </c>
       <c r="P36" s="36" t="n">
         <v>3</v>
       </c>
       <c r="Q36" s="38" t="s">
-        <v>270</v>
+        <v>304</v>
       </c>
       <c r="R36" s="36" t="s">
         <v>85</v>
@@ -8192,7 +8340,7 @@
     </row>
     <row r="37" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="41" t="s">
-        <v>271</v>
+        <v>305</v>
       </c>
       <c r="B37" s="42" t="n">
         <v>46318</v>
@@ -8204,13 +8352,13 @@
         <v>31</v>
       </c>
       <c r="E37" s="41" t="s">
-        <v>272</v>
+        <v>306</v>
       </c>
       <c r="F37" s="43" t="s">
-        <v>273</v>
+        <v>307</v>
       </c>
       <c r="G37" s="41" t="s">
-        <v>274</v>
+        <v>308</v>
       </c>
       <c r="H37" s="41" t="s">
         <v>80</v>
@@ -8219,7 +8367,7 @@
         <v>89</v>
       </c>
       <c r="J37" s="41" t="s">
-        <v>275</v>
+        <v>309</v>
       </c>
       <c r="K37" s="44" t="n">
         <v>55000</v>
@@ -8235,13 +8383,13 @@
         <v>43</v>
       </c>
       <c r="O37" s="45" t="s">
-        <v>83</v>
+        <v>310</v>
       </c>
       <c r="P37" s="41" t="n">
         <v>5</v>
       </c>
       <c r="Q37" s="43" t="s">
-        <v>276</v>
+        <v>311</v>
       </c>
       <c r="R37" s="41" t="s">
         <v>85</v>
@@ -8281,7 +8429,7 @@
     </row>
     <row r="38" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="36" t="s">
-        <v>277</v>
+        <v>312</v>
       </c>
       <c r="B38" s="37" t="n">
         <v>46318</v>
@@ -8293,13 +8441,13 @@
         <v>31</v>
       </c>
       <c r="E38" s="36" t="s">
-        <v>278</v>
+        <v>313</v>
       </c>
       <c r="F38" s="38" t="s">
-        <v>279</v>
+        <v>314</v>
       </c>
       <c r="G38" s="36" t="s">
-        <v>239</v>
+        <v>267</v>
       </c>
       <c r="H38" s="36" t="s">
         <v>80</v>
@@ -8308,7 +8456,7 @@
         <v>89</v>
       </c>
       <c r="J38" s="36" t="s">
-        <v>280</v>
+        <v>315</v>
       </c>
       <c r="K38" s="39" t="n">
         <v>65000</v>
@@ -8324,13 +8472,13 @@
         <v>43</v>
       </c>
       <c r="O38" s="40" t="s">
-        <v>83</v>
+        <v>316</v>
       </c>
       <c r="P38" s="36" t="n">
         <v>5</v>
       </c>
       <c r="Q38" s="38" t="s">
-        <v>281</v>
+        <v>317</v>
       </c>
       <c r="R38" s="36" t="s">
         <v>85</v>
@@ -8370,7 +8518,7 @@
     </row>
     <row r="39" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="41" t="s">
-        <v>282</v>
+        <v>318</v>
       </c>
       <c r="B39" s="42" t="n">
         <v>46318</v>
@@ -8382,13 +8530,13 @@
         <v>31</v>
       </c>
       <c r="E39" s="41" t="s">
-        <v>283</v>
+        <v>319</v>
       </c>
       <c r="F39" s="43" t="s">
-        <v>284</v>
+        <v>320</v>
       </c>
       <c r="G39" s="41" t="s">
-        <v>274</v>
+        <v>308</v>
       </c>
       <c r="H39" s="41" t="s">
         <v>80</v>
@@ -8397,7 +8545,7 @@
         <v>89</v>
       </c>
       <c r="J39" s="41" t="s">
-        <v>285</v>
+        <v>321</v>
       </c>
       <c r="K39" s="44" t="n">
         <v>77000</v>
@@ -8413,13 +8561,13 @@
         <v>43</v>
       </c>
       <c r="O39" s="45" t="s">
-        <v>83</v>
+        <v>322</v>
       </c>
       <c r="P39" s="41" t="n">
         <v>3</v>
       </c>
       <c r="Q39" s="43" t="s">
-        <v>286</v>
+        <v>323</v>
       </c>
       <c r="R39" s="41" t="s">
         <v>85</v>
@@ -8459,7 +8607,7 @@
     </row>
     <row r="40" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="36" t="s">
-        <v>287</v>
+        <v>324</v>
       </c>
       <c r="B40" s="37" t="n">
         <v>46318</v>
@@ -8471,13 +8619,13 @@
         <v>29</v>
       </c>
       <c r="E40" s="36" t="s">
-        <v>288</v>
+        <v>325</v>
       </c>
       <c r="F40" s="38" t="s">
-        <v>289</v>
+        <v>326</v>
       </c>
       <c r="G40" s="36" t="s">
-        <v>290</v>
+        <v>327</v>
       </c>
       <c r="H40" s="36" t="s">
         <v>80</v>
@@ -8486,7 +8634,7 @@
         <v>89</v>
       </c>
       <c r="J40" s="36" t="s">
-        <v>291</v>
+        <v>328</v>
       </c>
       <c r="K40" s="39" t="n">
         <v>70000</v>
@@ -8500,13 +8648,13 @@
         <v>43</v>
       </c>
       <c r="O40" s="40" t="s">
-        <v>83</v>
+        <v>329</v>
       </c>
       <c r="P40" s="36" t="n">
         <v>5</v>
       </c>
       <c r="Q40" s="38" t="s">
-        <v>292</v>
+        <v>330</v>
       </c>
       <c r="R40" s="36" t="s">
         <v>85</v>
@@ -8546,7 +8694,7 @@
     </row>
     <row r="41" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="41" t="s">
-        <v>293</v>
+        <v>331</v>
       </c>
       <c r="B41" s="42" t="n">
         <v>46318</v>
@@ -8558,13 +8706,13 @@
         <v>29</v>
       </c>
       <c r="E41" s="41" t="s">
-        <v>294</v>
+        <v>332</v>
       </c>
       <c r="F41" s="43" t="s">
-        <v>295</v>
+        <v>333</v>
       </c>
       <c r="G41" s="41" t="s">
-        <v>296</v>
+        <v>334</v>
       </c>
       <c r="H41" s="41" t="s">
         <v>80</v>
@@ -8573,7 +8721,7 @@
         <v>89</v>
       </c>
       <c r="J41" s="41" t="s">
-        <v>177</v>
+        <v>193</v>
       </c>
       <c r="K41" s="44" t="n">
         <v>80000</v>
@@ -8589,13 +8737,13 @@
         <v>43</v>
       </c>
       <c r="O41" s="45" t="s">
-        <v>83</v>
+        <v>335</v>
       </c>
       <c r="P41" s="41" t="n">
         <v>3</v>
       </c>
       <c r="Q41" s="43" t="s">
-        <v>297</v>
+        <v>336</v>
       </c>
       <c r="R41" s="41" t="s">
         <v>85</v>
@@ -8635,7 +8783,7 @@
     </row>
     <row r="42" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="36" t="s">
-        <v>298</v>
+        <v>337</v>
       </c>
       <c r="B42" s="37" t="n">
         <v>46318</v>
@@ -8647,13 +8795,13 @@
         <v>31</v>
       </c>
       <c r="E42" s="36" t="s">
-        <v>299</v>
+        <v>338</v>
       </c>
       <c r="F42" s="38" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="G42" s="36" t="s">
-        <v>300</v>
+        <v>339</v>
       </c>
       <c r="H42" s="36" t="s">
         <v>80</v>
@@ -8662,7 +8810,7 @@
         <v>89</v>
       </c>
       <c r="J42" s="36" t="s">
-        <v>301</v>
+        <v>340</v>
       </c>
       <c r="K42" s="39" t="n">
         <v>85000</v>
@@ -8678,13 +8826,13 @@
         <v>43</v>
       </c>
       <c r="O42" s="40" t="s">
-        <v>83</v>
+        <v>341</v>
       </c>
       <c r="P42" s="36" t="n">
         <v>3</v>
       </c>
       <c r="Q42" s="38" t="s">
-        <v>302</v>
+        <v>342</v>
       </c>
       <c r="R42" s="36" t="s">
         <v>85</v>
@@ -8724,7 +8872,7 @@
     </row>
     <row r="43" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="41" t="s">
-        <v>303</v>
+        <v>343</v>
       </c>
       <c r="B43" s="42" t="n">
         <v>46318</v>
@@ -8736,13 +8884,13 @@
         <v>34</v>
       </c>
       <c r="E43" s="41" t="s">
-        <v>304</v>
+        <v>344</v>
       </c>
       <c r="F43" s="43" t="s">
-        <v>305</v>
+        <v>345</v>
       </c>
       <c r="G43" s="41" t="s">
-        <v>306</v>
+        <v>346</v>
       </c>
       <c r="H43" s="41" t="s">
         <v>80</v>
@@ -8751,7 +8899,7 @@
         <v>89</v>
       </c>
       <c r="J43" s="41" t="s">
-        <v>307</v>
+        <v>347</v>
       </c>
       <c r="K43" s="44" t="n">
         <v>70600</v>
@@ -8767,13 +8915,13 @@
         <v>43</v>
       </c>
       <c r="O43" s="45" t="s">
-        <v>83</v>
+        <v>348</v>
       </c>
       <c r="P43" s="41" t="n">
         <v>5</v>
       </c>
       <c r="Q43" s="43" t="s">
-        <v>308</v>
+        <v>349</v>
       </c>
       <c r="R43" s="41" t="s">
         <v>85</v>
@@ -8813,7 +8961,7 @@
     </row>
     <row r="44" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="36" t="s">
-        <v>309</v>
+        <v>350</v>
       </c>
       <c r="B44" s="37" t="n">
         <v>46318</v>
@@ -8825,13 +8973,13 @@
         <v>34</v>
       </c>
       <c r="E44" s="36" t="s">
-        <v>310</v>
+        <v>351</v>
       </c>
       <c r="F44" s="38" t="s">
-        <v>311</v>
+        <v>352</v>
       </c>
       <c r="G44" s="36" t="s">
-        <v>256</v>
+        <v>287</v>
       </c>
       <c r="H44" s="36" t="s">
         <v>80</v>
@@ -8840,7 +8988,7 @@
         <v>89</v>
       </c>
       <c r="J44" s="36" t="s">
-        <v>312</v>
+        <v>353</v>
       </c>
       <c r="K44" s="39" t="n">
         <v>105000</v>
@@ -8856,13 +9004,13 @@
         <v>43</v>
       </c>
       <c r="O44" s="40" t="s">
-        <v>83</v>
+        <v>354</v>
       </c>
       <c r="P44" s="36" t="n">
         <v>3</v>
       </c>
       <c r="Q44" s="38" t="s">
-        <v>313</v>
+        <v>355</v>
       </c>
       <c r="R44" s="36" t="s">
         <v>85</v>
@@ -8902,7 +9050,7 @@
     </row>
     <row r="45" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="41" t="s">
-        <v>314</v>
+        <v>356</v>
       </c>
       <c r="B45" s="42" t="n">
         <v>46318</v>
@@ -8914,13 +9062,13 @@
         <v>34</v>
       </c>
       <c r="E45" s="41" t="s">
-        <v>315</v>
+        <v>357</v>
       </c>
       <c r="F45" s="43" t="s">
-        <v>316</v>
+        <v>358</v>
       </c>
       <c r="G45" s="41" t="s">
-        <v>306</v>
+        <v>346</v>
       </c>
       <c r="H45" s="41" t="s">
         <v>80</v>
@@ -8929,7 +9077,7 @@
         <v>89</v>
       </c>
       <c r="J45" s="41" t="s">
-        <v>317</v>
+        <v>359</v>
       </c>
       <c r="K45" s="44" t="n">
         <v>56615</v>
@@ -8945,13 +9093,13 @@
         <v>43</v>
       </c>
       <c r="O45" s="45" t="s">
-        <v>83</v>
+        <v>360</v>
       </c>
       <c r="P45" s="41" t="n">
         <v>3</v>
       </c>
       <c r="Q45" s="43" t="s">
-        <v>318</v>
+        <v>361</v>
       </c>
       <c r="R45" s="41" t="s">
         <v>85</v>
@@ -8991,7 +9139,7 @@
     </row>
     <row r="46" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="36" t="s">
-        <v>319</v>
+        <v>362</v>
       </c>
       <c r="B46" s="37" t="n">
         <v>46318</v>
@@ -9003,13 +9151,13 @@
         <v>34</v>
       </c>
       <c r="E46" s="36" t="s">
-        <v>320</v>
+        <v>363</v>
       </c>
       <c r="F46" s="38" t="s">
-        <v>321</v>
+        <v>364</v>
       </c>
       <c r="G46" s="36" t="s">
-        <v>322</v>
+        <v>365</v>
       </c>
       <c r="H46" s="36" t="s">
         <v>80</v>
@@ -9018,7 +9166,7 @@
         <v>89</v>
       </c>
       <c r="J46" s="36" t="s">
-        <v>323</v>
+        <v>366</v>
       </c>
       <c r="K46" s="39" t="n">
         <v>65000</v>
@@ -9034,13 +9182,13 @@
         <v>43</v>
       </c>
       <c r="O46" s="40" t="s">
-        <v>83</v>
+        <v>367</v>
       </c>
       <c r="P46" s="36" t="n">
         <v>3</v>
       </c>
       <c r="Q46" s="38" t="s">
-        <v>324</v>
+        <v>368</v>
       </c>
       <c r="R46" s="36" t="s">
         <v>85</v>
@@ -9080,7 +9228,7 @@
     </row>
     <row r="47" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="41" t="s">
-        <v>325</v>
+        <v>369</v>
       </c>
       <c r="B47" s="42" t="n">
         <v>46318</v>
@@ -9092,13 +9240,13 @@
         <v>34</v>
       </c>
       <c r="E47" s="41" t="s">
-        <v>326</v>
+        <v>370</v>
       </c>
       <c r="F47" s="43" t="s">
-        <v>327</v>
+        <v>371</v>
       </c>
       <c r="G47" s="41" t="s">
-        <v>239</v>
+        <v>267</v>
       </c>
       <c r="H47" s="41" t="s">
         <v>80</v>
@@ -9107,7 +9255,7 @@
         <v>89</v>
       </c>
       <c r="J47" s="41" t="s">
-        <v>328</v>
+        <v>372</v>
       </c>
       <c r="K47" s="44" t="n">
         <v>89600</v>
@@ -9123,13 +9271,13 @@
         <v>43</v>
       </c>
       <c r="O47" s="45" t="s">
-        <v>83</v>
+        <v>373</v>
       </c>
       <c r="P47" s="41" t="n">
         <v>3</v>
       </c>
       <c r="Q47" s="43" t="s">
-        <v>329</v>
+        <v>374</v>
       </c>
       <c r="R47" s="41" t="s">
         <v>85</v>
@@ -9169,7 +9317,7 @@
     </row>
     <row r="48" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="36" t="s">
-        <v>330</v>
+        <v>375</v>
       </c>
       <c r="B48" s="37" t="n">
         <v>46318</v>
@@ -9181,13 +9329,13 @@
         <v>31</v>
       </c>
       <c r="E48" s="36" t="s">
-        <v>331</v>
+        <v>376</v>
       </c>
       <c r="F48" s="38" t="s">
-        <v>332</v>
+        <v>377</v>
       </c>
       <c r="G48" s="36" t="s">
-        <v>333</v>
+        <v>378</v>
       </c>
       <c r="H48" s="36" t="s">
         <v>80</v>
@@ -9196,7 +9344,7 @@
         <v>89</v>
       </c>
       <c r="J48" s="36" t="s">
-        <v>334</v>
+        <v>379</v>
       </c>
       <c r="K48" s="39" t="n">
         <v>58000</v>
@@ -9212,13 +9360,13 @@
         <v>43</v>
       </c>
       <c r="O48" s="40" t="s">
-        <v>83</v>
+        <v>380</v>
       </c>
       <c r="P48" s="36" t="n">
         <v>5</v>
       </c>
       <c r="Q48" s="38" t="s">
-        <v>335</v>
+        <v>381</v>
       </c>
       <c r="R48" s="36" t="s">
         <v>85</v>
@@ -9258,7 +9406,7 @@
     </row>
     <row r="49" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="41" t="s">
-        <v>336</v>
+        <v>382</v>
       </c>
       <c r="B49" s="42" t="n">
         <v>46318</v>
@@ -9270,22 +9418,22 @@
         <v>31</v>
       </c>
       <c r="E49" s="41" t="s">
-        <v>337</v>
+        <v>383</v>
       </c>
       <c r="F49" s="43" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G49" s="41" t="s">
-        <v>338</v>
+        <v>384</v>
       </c>
       <c r="H49" s="41" t="s">
         <v>80</v>
       </c>
       <c r="I49" s="41" t="s">
-        <v>339</v>
+        <v>385</v>
       </c>
       <c r="J49" s="41" t="s">
-        <v>340</v>
+        <v>386</v>
       </c>
       <c r="K49" s="44" t="n">
         <v>52000</v>
@@ -9301,13 +9449,13 @@
         <v>43</v>
       </c>
       <c r="O49" s="45" t="s">
-        <v>83</v>
+        <v>387</v>
       </c>
       <c r="P49" s="41" t="n">
         <v>3</v>
       </c>
       <c r="Q49" s="43" t="s">
-        <v>341</v>
+        <v>388</v>
       </c>
       <c r="R49" s="41" t="s">
         <v>85</v>
@@ -9347,7 +9495,7 @@
     </row>
     <row r="50" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="36" t="s">
-        <v>342</v>
+        <v>389</v>
       </c>
       <c r="B50" s="37" t="n">
         <v>46318</v>
@@ -9359,13 +9507,13 @@
         <v>31</v>
       </c>
       <c r="E50" s="36" t="s">
-        <v>343</v>
+        <v>390</v>
       </c>
       <c r="F50" s="38" t="s">
-        <v>344</v>
+        <v>391</v>
       </c>
       <c r="G50" s="36" t="s">
-        <v>345</v>
+        <v>392</v>
       </c>
       <c r="H50" s="36" t="s">
         <v>80</v>
@@ -9374,7 +9522,7 @@
         <v>89</v>
       </c>
       <c r="J50" s="36" t="s">
-        <v>346</v>
+        <v>393</v>
       </c>
       <c r="K50" s="39" t="n">
         <v>75000</v>
@@ -9388,13 +9536,13 @@
         <v>43</v>
       </c>
       <c r="O50" s="40" t="s">
-        <v>83</v>
+        <v>394</v>
       </c>
       <c r="P50" s="36" t="n">
         <v>3</v>
       </c>
       <c r="Q50" s="38" t="s">
-        <v>347</v>
+        <v>395</v>
       </c>
       <c r="R50" s="36" t="s">
         <v>85</v>
@@ -9434,7 +9582,7 @@
     </row>
     <row r="51" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="41" t="s">
-        <v>348</v>
+        <v>396</v>
       </c>
       <c r="B51" s="42" t="n">
         <v>46318</v>
@@ -9446,13 +9594,13 @@
         <v>31</v>
       </c>
       <c r="E51" s="41" t="s">
-        <v>349</v>
+        <v>397</v>
       </c>
       <c r="F51" s="43" t="s">
-        <v>273</v>
+        <v>307</v>
       </c>
       <c r="G51" s="41" t="s">
-        <v>350</v>
+        <v>398</v>
       </c>
       <c r="H51" s="41" t="s">
         <v>80</v>
@@ -9461,7 +9609,7 @@
         <v>89</v>
       </c>
       <c r="J51" s="41" t="s">
-        <v>351</v>
+        <v>399</v>
       </c>
       <c r="K51" s="44" t="n">
         <v>83200</v>
@@ -9477,13 +9625,13 @@
         <v>43</v>
       </c>
       <c r="O51" s="45" t="s">
-        <v>83</v>
+        <v>400</v>
       </c>
       <c r="P51" s="41" t="n">
         <v>3</v>
       </c>
       <c r="Q51" s="43" t="s">
-        <v>352</v>
+        <v>401</v>
       </c>
       <c r="R51" s="41" t="s">
         <v>85</v>
@@ -9621,56 +9769,56 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="O2" r:id="rId1" display="Apply ↗"/>
-    <hyperlink ref="O3" r:id="rId2" display="Apply ↗"/>
-    <hyperlink ref="O4" r:id="rId3" display="Apply ↗"/>
-    <hyperlink ref="O5" r:id="rId4" display="Apply ↗"/>
-    <hyperlink ref="O6" r:id="rId5" display="Apply ↗"/>
-    <hyperlink ref="O7" r:id="rId6" display="Apply ↗"/>
-    <hyperlink ref="O8" r:id="rId7" display="Apply ↗"/>
-    <hyperlink ref="O9" r:id="rId8" display="Apply ↗"/>
-    <hyperlink ref="O10" r:id="rId9" display="Apply ↗"/>
-    <hyperlink ref="O11" r:id="rId10" display="Apply ↗"/>
-    <hyperlink ref="O12" r:id="rId11" display="Apply ↗"/>
-    <hyperlink ref="O13" r:id="rId12" display="Apply ↗"/>
-    <hyperlink ref="O14" r:id="rId13" display="Apply ↗"/>
-    <hyperlink ref="O15" r:id="rId14" display="Apply ↗"/>
-    <hyperlink ref="O16" r:id="rId15" display="Apply ↗"/>
-    <hyperlink ref="O17" r:id="rId16" display="Apply ↗"/>
-    <hyperlink ref="O18" r:id="rId17" display="Apply ↗"/>
-    <hyperlink ref="O19" r:id="rId18" display="Apply ↗"/>
-    <hyperlink ref="O20" r:id="rId19" display="Apply ↗"/>
-    <hyperlink ref="O21" r:id="rId20" display="Apply ↗"/>
-    <hyperlink ref="O22" r:id="rId21" display="Apply ↗"/>
-    <hyperlink ref="O23" r:id="rId22" display="Apply ↗"/>
-    <hyperlink ref="O24" r:id="rId23" display="Apply ↗"/>
-    <hyperlink ref="O25" r:id="rId24" display="Apply ↗"/>
-    <hyperlink ref="O26" r:id="rId25" display="Apply ↗"/>
-    <hyperlink ref="O27" r:id="rId26" display="Apply ↗"/>
-    <hyperlink ref="O28" r:id="rId27" display="Apply ↗"/>
-    <hyperlink ref="O29" r:id="rId28" display="Apply ↗"/>
-    <hyperlink ref="O30" r:id="rId29" display="Apply ↗"/>
-    <hyperlink ref="O31" r:id="rId30" display="Apply ↗"/>
-    <hyperlink ref="O32" r:id="rId31" display="Apply ↗"/>
-    <hyperlink ref="O33" r:id="rId32" display="Apply ↗"/>
-    <hyperlink ref="O34" r:id="rId33" display="Apply ↗"/>
-    <hyperlink ref="O35" r:id="rId34" display="Apply ↗"/>
-    <hyperlink ref="O36" r:id="rId35" display="Apply ↗"/>
-    <hyperlink ref="O37" r:id="rId36" display="Apply ↗"/>
-    <hyperlink ref="O38" r:id="rId37" display="Apply ↗"/>
-    <hyperlink ref="O39" r:id="rId38" display="Apply ↗"/>
-    <hyperlink ref="O40" r:id="rId39" display="Apply ↗"/>
-    <hyperlink ref="O41" r:id="rId40" display="Apply ↗"/>
-    <hyperlink ref="O42" r:id="rId41" display="Apply ↗"/>
-    <hyperlink ref="O43" r:id="rId42" display="Apply ↗"/>
-    <hyperlink ref="O44" r:id="rId43" display="Apply ↗"/>
-    <hyperlink ref="O45" r:id="rId44" display="Apply ↗"/>
-    <hyperlink ref="O46" r:id="rId45" display="Apply ↗"/>
-    <hyperlink ref="O47" r:id="rId46" display="Apply ↗"/>
-    <hyperlink ref="O48" r:id="rId47" display="Apply ↗"/>
-    <hyperlink ref="O49" r:id="rId48" display="Apply ↗"/>
-    <hyperlink ref="O50" r:id="rId49" display="Apply ↗"/>
-    <hyperlink ref="O51" r:id="rId50" display="Apply ↗"/>
+    <hyperlink ref="O2" r:id="rId1" display="https://to.indeed.com/aax99gw6hbrb"/>
+    <hyperlink ref="O3" r:id="rId2" display="https://to.indeed.com/aay7xrszvfcz"/>
+    <hyperlink ref="O4" r:id="rId3" display="https://to.indeed.com/aavpsvxl96nc"/>
+    <hyperlink ref="O5" r:id="rId4" display="https://to.indeed.com/aa7fjmb4wpj2"/>
+    <hyperlink ref="O6" r:id="rId5" display="https://to.indeed.com/aacwsr2qtwlb"/>
+    <hyperlink ref="O7" r:id="rId6" display="https://to.indeed.com/aal4dgvq6xv9"/>
+    <hyperlink ref="O8" r:id="rId7" display="https://to.indeed.com/aajvsvfvjwrc"/>
+    <hyperlink ref="O9" r:id="rId8" display="https://to.indeed.com/aaps72t8dk8f"/>
+    <hyperlink ref="O10" r:id="rId9" display="https://to.indeed.com/aa2qxtmxy4bd"/>
+    <hyperlink ref="O11" r:id="rId10" display="https://to.indeed.com/aads28mmkhyq"/>
+    <hyperlink ref="O12" r:id="rId11" display="https://to.indeed.com/aa7g6jc9nyk9"/>
+    <hyperlink ref="O13" r:id="rId12" display="https://to.indeed.com/aavdnzl4qqkf"/>
+    <hyperlink ref="O14" r:id="rId13" display="https://to.indeed.com/aa7r9mwd7n4z"/>
+    <hyperlink ref="O15" r:id="rId14" display="https://to.indeed.com/aay7qpqwv4hm"/>
+    <hyperlink ref="O16" r:id="rId15" display="https://to.indeed.com/aajzj8rzxsjj"/>
+    <hyperlink ref="O17" r:id="rId16" display="https://to.indeed.com/aaygkdv8pht9"/>
+    <hyperlink ref="O18" r:id="rId17" display="https://to.indeed.com/aa4gbvpbhrlr"/>
+    <hyperlink ref="O19" r:id="rId18" display="https://to.indeed.com/aabjzr679tlv"/>
+    <hyperlink ref="O20" r:id="rId19" display="https://to.indeed.com/aa4kgd6sbtmp"/>
+    <hyperlink ref="O21" r:id="rId20" display="https://to.indeed.com/aatfz6q9xtf4"/>
+    <hyperlink ref="O22" r:id="rId21" display="https://to.indeed.com/aay22djqkzs4"/>
+    <hyperlink ref="O23" r:id="rId22" display="https://to.indeed.com/aaph7dxt762l"/>
+    <hyperlink ref="O24" r:id="rId23" display="https://to.indeed.com/aaqvns2cnd8q"/>
+    <hyperlink ref="O25" r:id="rId24" display="https://to.indeed.com/aagzwvczrjsl"/>
+    <hyperlink ref="O26" r:id="rId25" display="https://to.indeed.com/aagnx8j42zdy"/>
+    <hyperlink ref="O27" r:id="rId26" display="https://to.indeed.com/aakg8s2nsqlb"/>
+    <hyperlink ref="O28" r:id="rId27" display="https://to.indeed.com/aa4k6ln4yhdj"/>
+    <hyperlink ref="O29" r:id="rId28" display="https://to.indeed.com/aay8bxlp2jhm"/>
+    <hyperlink ref="O30" r:id="rId29" display="https://to.indeed.com/aa6bykh42c27"/>
+    <hyperlink ref="O31" r:id="rId30" display="https://to.indeed.com/aarswx9rsgg8"/>
+    <hyperlink ref="O32" r:id="rId31" display="https://to.indeed.com/aaszbvtnmqgd"/>
+    <hyperlink ref="O33" r:id="rId32" display="https://to.indeed.com/aazrgznjy9nf"/>
+    <hyperlink ref="O34" r:id="rId33" display="https://to.indeed.com/aar9jthdmd6m"/>
+    <hyperlink ref="O35" r:id="rId34" display="https://to.indeed.com/aahggs7qsv2t"/>
+    <hyperlink ref="O36" r:id="rId35" display="https://to.indeed.com/aabxzz7wbksg"/>
+    <hyperlink ref="O37" r:id="rId36" display="https://to.indeed.com/aa7bgbfgdsvq"/>
+    <hyperlink ref="O38" r:id="rId37" display="https://to.indeed.com/aagcmn2bgpkl"/>
+    <hyperlink ref="O39" r:id="rId38" display="https://to.indeed.com/aa6kytzgsfc9"/>
+    <hyperlink ref="O40" r:id="rId39" display="https://to.indeed.com/aa2kp46gqspf"/>
+    <hyperlink ref="O41" r:id="rId40" display="https://to.indeed.com/aaxvy66h9pbv"/>
+    <hyperlink ref="O42" r:id="rId41" display="https://to.indeed.com/aajwldks9z8f"/>
+    <hyperlink ref="O43" r:id="rId42" display="https://to.indeed.com/aaqcrksckysy"/>
+    <hyperlink ref="O44" r:id="rId43" display="https://to.indeed.com/aap2xlmscfpk"/>
+    <hyperlink ref="O45" r:id="rId44" display="https://to.indeed.com/aamzf2mnbbvv"/>
+    <hyperlink ref="O46" r:id="rId45" display="https://to.indeed.com/aarjzv4yn92x"/>
+    <hyperlink ref="O47" r:id="rId46" display="https://to.indeed.com/aa46td7q2glh"/>
+    <hyperlink ref="O48" r:id="rId47" display="https://to.indeed.com/aa2gprnx4j7z"/>
+    <hyperlink ref="O49" r:id="rId48" display="https://to.indeed.com/aa6fwcg78vsx"/>
+    <hyperlink ref="O50" r:id="rId49" display="https://to.indeed.com/aajxwjry2ssr"/>
+    <hyperlink ref="O51" r:id="rId50" display="https://to.indeed.com/aa4q4nmv9jr6"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -9718,7 +9866,7 @@
         <v>53</v>
       </c>
       <c r="D1" s="46" t="s">
-        <v>353</v>
+        <v>402</v>
       </c>
       <c r="E1" s="46" t="s">
         <v>65</v>
@@ -9742,13 +9890,13 @@
         <v>68</v>
       </c>
       <c r="L1" s="46" t="s">
-        <v>354</v>
+        <v>403</v>
       </c>
       <c r="M1" s="46" t="s">
         <v>70</v>
       </c>
       <c r="N1" s="46" t="s">
-        <v>355</v>
+        <v>404</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21440,7 +21588,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="47" t="s">
-        <v>356</v>
+        <v>405</v>
       </c>
       <c r="B1" s="47"/>
       <c r="C1" s="47"/>
@@ -21451,22 +21599,22 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="48" t="s">
-        <v>357</v>
+        <v>406</v>
       </c>
       <c r="B2" s="48" t="s">
         <v>49</v>
       </c>
       <c r="C2" s="48" t="s">
-        <v>358</v>
+        <v>407</v>
       </c>
       <c r="D2" s="48" t="s">
-        <v>359</v>
+        <v>408</v>
       </c>
       <c r="E2" s="48" t="s">
-        <v>360</v>
+        <v>409</v>
       </c>
       <c r="F2" s="48" t="s">
-        <v>361</v>
+        <v>410</v>
       </c>
       <c r="G2" s="48" t="s">
         <v>69</v>
@@ -21484,13 +21632,13 @@
         <v>Feature Solutions</v>
       </c>
       <c r="D3" s="41" t="s">
-        <v>362</v>
+        <v>411</v>
       </c>
       <c r="E3" s="50" t="s">
-        <v>363</v>
+        <v>412</v>
       </c>
       <c r="F3" s="41" t="s">
-        <v>364</v>
+        <v>413</v>
       </c>
       <c r="G3" s="42" t="n">
         <v>46321</v>
@@ -24507,7 +24655,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="51" t="s">
-        <v>365</v>
+        <v>414</v>
       </c>
       <c r="B1" s="51"/>
       <c r="C1" s="51"/>
@@ -24522,48 +24670,48 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="52" t="s">
-        <v>366</v>
+        <v>415</v>
       </c>
       <c r="B2" s="52" t="s">
         <v>52</v>
       </c>
       <c r="C2" s="52" t="s">
-        <v>367</v>
+        <v>416</v>
       </c>
       <c r="D2" s="52" t="s">
         <v>49</v>
       </c>
       <c r="E2" s="52" t="s">
-        <v>368</v>
+        <v>417</v>
       </c>
       <c r="F2" s="52" t="s">
-        <v>369</v>
+        <v>418</v>
       </c>
       <c r="G2" s="52" t="s">
-        <v>370</v>
+        <v>419</v>
       </c>
       <c r="H2" s="52" t="s">
         <v>66</v>
       </c>
       <c r="I2" s="52" t="s">
-        <v>361</v>
+        <v>410</v>
       </c>
       <c r="J2" s="52" t="s">
         <v>69</v>
       </c>
       <c r="K2" s="52" t="s">
-        <v>360</v>
+        <v>409</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="49" t="s">
-        <v>371</v>
+        <v>420</v>
       </c>
       <c r="B3" s="41" t="s">
         <v>87</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>372</v>
+        <v>421</v>
       </c>
       <c r="D3" s="41" t="s">
         <v>86</v>
@@ -24576,16 +24724,16 @@
         <v>46319</v>
       </c>
       <c r="H3" s="41" t="s">
-        <v>373</v>
+        <v>422</v>
       </c>
       <c r="I3" s="41" t="s">
-        <v>374</v>
+        <v>423</v>
       </c>
       <c r="J3" s="42" t="n">
         <v>46326</v>
       </c>
       <c r="K3" s="50" t="s">
-        <v>375</v>
+        <v>424</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26545,7 +26693,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="53" t="s">
-        <v>376</v>
+        <v>425</v>
       </c>
       <c r="B1" s="53"/>
       <c r="C1" s="53"/>
@@ -26554,7 +26702,7 @@
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="54" t="s">
-        <v>377</v>
+        <v>426</v>
       </c>
       <c r="B2" s="54"/>
       <c r="C2" s="54"/>
@@ -26563,230 +26711,230 @@
     </row>
     <row r="4" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="55" t="s">
-        <v>378</v>
+        <v>427</v>
       </c>
       <c r="B4" s="55"/>
       <c r="D4" s="56" t="s">
-        <v>379</v>
+        <v>428</v>
       </c>
       <c r="E4" s="56"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="57" t="s">
-        <v>380</v>
+        <v>429</v>
       </c>
       <c r="B5" s="57" t="s">
-        <v>381</v>
+        <v>430</v>
       </c>
       <c r="D5" s="58" t="s">
-        <v>380</v>
+        <v>429</v>
       </c>
       <c r="E5" s="58" t="s">
-        <v>381</v>
+        <v>430</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="59" t="s">
-        <v>382</v>
+        <v>431</v>
       </c>
       <c r="B6" s="60" t="s">
-        <v>383</v>
+        <v>432</v>
       </c>
       <c r="D6" s="61" t="s">
-        <v>384</v>
+        <v>433</v>
       </c>
       <c r="E6" s="60" t="s">
-        <v>385</v>
+        <v>434</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="59" t="s">
-        <v>386</v>
+        <v>435</v>
       </c>
       <c r="B7" s="60" t="s">
-        <v>387</v>
+        <v>436</v>
       </c>
       <c r="D7" s="61" t="s">
-        <v>388</v>
+        <v>437</v>
       </c>
       <c r="E7" s="60" t="s">
-        <v>389</v>
+        <v>438</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="59" t="s">
-        <v>390</v>
+        <v>439</v>
       </c>
       <c r="B8" s="60" t="s">
-        <v>391</v>
+        <v>440</v>
       </c>
       <c r="D8" s="61" t="s">
-        <v>392</v>
+        <v>441</v>
       </c>
       <c r="E8" s="60" t="s">
-        <v>393</v>
+        <v>442</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="59" t="s">
-        <v>394</v>
+        <v>443</v>
       </c>
       <c r="B9" s="60" t="s">
-        <v>395</v>
+        <v>444</v>
       </c>
       <c r="D9" s="61" t="s">
-        <v>396</v>
+        <v>445</v>
       </c>
       <c r="E9" s="60" t="s">
-        <v>397</v>
+        <v>446</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="59" t="s">
-        <v>398</v>
+        <v>447</v>
       </c>
       <c r="B10" s="60" t="s">
-        <v>399</v>
+        <v>448</v>
       </c>
       <c r="D10" s="61" t="s">
-        <v>400</v>
+        <v>449</v>
       </c>
       <c r="E10" s="60" t="s">
-        <v>401</v>
+        <v>450</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="59" t="s">
-        <v>402</v>
+        <v>451</v>
       </c>
       <c r="B11" s="60" t="s">
-        <v>403</v>
+        <v>452</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="59" t="s">
-        <v>404</v>
+        <v>453</v>
       </c>
       <c r="B12" s="60" t="s">
-        <v>405</v>
+        <v>454</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="59" t="s">
-        <v>406</v>
+        <v>455</v>
       </c>
       <c r="B13" s="60" t="s">
-        <v>407</v>
+        <v>456</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="59" t="s">
-        <v>408</v>
+        <v>457</v>
       </c>
       <c r="B14" s="60" t="s">
-        <v>409</v>
+        <v>458</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="62" t="s">
-        <v>410</v>
+        <v>459</v>
       </c>
       <c r="B16" s="62"/>
       <c r="D16" s="63" t="s">
-        <v>411</v>
+        <v>460</v>
       </c>
       <c r="E16" s="63"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="64" t="s">
-        <v>380</v>
+        <v>429</v>
       </c>
       <c r="B17" s="64" t="s">
-        <v>381</v>
+        <v>430</v>
       </c>
       <c r="D17" s="65" t="s">
-        <v>380</v>
+        <v>429</v>
       </c>
       <c r="E17" s="65" t="s">
-        <v>381</v>
+        <v>430</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="66" t="s">
-        <v>412</v>
+        <v>461</v>
       </c>
       <c r="B18" s="60" t="s">
-        <v>413</v>
+        <v>462</v>
       </c>
       <c r="D18" s="67" t="s">
-        <v>414</v>
+        <v>463</v>
       </c>
       <c r="E18" s="60" t="s">
-        <v>415</v>
+        <v>464</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="66" t="s">
-        <v>416</v>
+        <v>465</v>
       </c>
       <c r="B19" s="60" t="s">
-        <v>417</v>
+        <v>466</v>
       </c>
       <c r="D19" s="67" t="s">
-        <v>418</v>
+        <v>467</v>
       </c>
       <c r="E19" s="60" t="s">
-        <v>419</v>
+        <v>468</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="66" t="s">
-        <v>420</v>
+        <v>469</v>
       </c>
       <c r="B20" s="60" t="s">
-        <v>421</v>
+        <v>470</v>
       </c>
       <c r="D20" s="67" t="s">
-        <v>422</v>
+        <v>471</v>
       </c>
       <c r="E20" s="60" t="s">
-        <v>423</v>
+        <v>472</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="66" t="s">
-        <v>424</v>
+        <v>473</v>
       </c>
       <c r="B21" s="60" t="s">
-        <v>425</v>
+        <v>474</v>
       </c>
       <c r="D21" s="67" t="s">
-        <v>426</v>
+        <v>475</v>
       </c>
       <c r="E21" s="60" t="s">
-        <v>427</v>
+        <v>476</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="66" t="s">
-        <v>428</v>
+        <v>477</v>
       </c>
       <c r="B22" s="60" t="s">
-        <v>429</v>
+        <v>478</v>
       </c>
       <c r="D22" s="67" t="s">
-        <v>430</v>
+        <v>479</v>
       </c>
       <c r="E22" s="60" t="s">
-        <v>431</v>
+        <v>480</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="66" t="s">
-        <v>432</v>
+        <v>481</v>
       </c>
       <c r="B23" s="60" t="s">
-        <v>433</v>
+        <v>482</v>
       </c>
     </row>
   </sheetData>
@@ -26833,48 +26981,48 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="68" t="s">
-        <v>434</v>
+        <v>483</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="35" t="s">
-        <v>435</v>
+        <v>484</v>
       </c>
       <c r="B2" s="35" t="s">
-        <v>436</v>
+        <v>485</v>
       </c>
       <c r="C2" s="35" t="s">
-        <v>437</v>
+        <v>486</v>
       </c>
       <c r="D2" s="35" t="s">
-        <v>438</v>
+        <v>487</v>
       </c>
       <c r="E2" s="35" t="s">
-        <v>439</v>
+        <v>488</v>
       </c>
       <c r="F2" s="35" t="s">
-        <v>440</v>
+        <v>489</v>
       </c>
       <c r="G2" s="35" t="s">
-        <v>441</v>
+        <v>490</v>
       </c>
       <c r="H2" s="35" t="s">
-        <v>442</v>
+        <v>491</v>
       </c>
       <c r="I2" s="35" t="s">
-        <v>443</v>
+        <v>492</v>
       </c>
       <c r="J2" s="35" t="s">
         <v>41</v>
       </c>
       <c r="K2" s="35" t="s">
-        <v>444</v>
+        <v>493</v>
       </c>
       <c r="L2" s="35" t="s">
-        <v>445</v>
+        <v>494</v>
       </c>
       <c r="M2" s="35" t="s">
-        <v>446</v>
+        <v>495</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26897,25 +27045,25 @@
         <v>1</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>447</v>
+        <v>496</v>
       </c>
       <c r="H3" s="13" t="s">
         <v>85</v>
       </c>
       <c r="I3" s="13" t="s">
-        <v>362</v>
+        <v>411</v>
       </c>
       <c r="J3" s="13" t="s">
-        <v>373</v>
+        <v>422</v>
       </c>
       <c r="K3" s="13" t="s">
         <v>45</v>
       </c>
       <c r="L3" s="13" t="s">
-        <v>448</v>
+        <v>497</v>
       </c>
       <c r="M3" s="13" t="s">
-        <v>364</v>
+        <v>413</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26926,7 +27074,7 @@
         <v>8</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>233</v>
+        <v>260</v>
       </c>
       <c r="D4" s="13" t="s">
         <v>81</v>
@@ -26938,25 +27086,25 @@
         <v>2</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>449</v>
+        <v>498</v>
       </c>
       <c r="H4" s="13" t="s">
-        <v>450</v>
+        <v>499</v>
       </c>
       <c r="I4" s="13" t="s">
         <v>8</v>
       </c>
       <c r="J4" s="13" t="s">
-        <v>451</v>
+        <v>500</v>
       </c>
       <c r="K4" s="13" t="s">
-        <v>452</v>
+        <v>501</v>
       </c>
       <c r="L4" s="13" t="s">
-        <v>453</v>
+        <v>502</v>
       </c>
       <c r="M4" s="13" t="s">
-        <v>454</v>
+        <v>503</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26967,10 +27115,10 @@
         <v>16</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>455</v>
+        <v>504</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>456</v>
+        <v>505</v>
       </c>
       <c r="E5" s="13" t="s">
         <v>45</v>
@@ -26979,22 +27127,22 @@
         <v>3</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="I5" s="13" t="s">
-        <v>457</v>
+        <v>506</v>
       </c>
       <c r="J5" s="13" t="s">
-        <v>458</v>
+        <v>507</v>
       </c>
       <c r="K5" s="13" t="s">
-        <v>459</v>
+        <v>508</v>
       </c>
       <c r="L5" s="13" t="s">
-        <v>460</v>
+        <v>509</v>
       </c>
       <c r="M5" s="13" t="s">
-        <v>374</v>
+        <v>423</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27005,10 +27153,10 @@
         <v>17</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>461</v>
+        <v>510</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>339</v>
+        <v>385</v>
       </c>
       <c r="E6" s="13" t="s">
         <v>46</v>
@@ -27017,22 +27165,22 @@
         <v>4</v>
       </c>
       <c r="H6" s="13" t="s">
-        <v>462</v>
+        <v>511</v>
       </c>
       <c r="I6" s="13" t="s">
-        <v>463</v>
+        <v>512</v>
       </c>
       <c r="J6" s="13" t="s">
-        <v>464</v>
+        <v>513</v>
       </c>
       <c r="K6" s="13" t="s">
-        <v>465</v>
+        <v>514</v>
       </c>
       <c r="L6" s="13" t="s">
-        <v>466</v>
+        <v>515</v>
       </c>
       <c r="M6" s="13" t="s">
-        <v>467</v>
+        <v>516</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27043,7 +27191,7 @@
         <v>18</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>206</v>
+        <v>228</v>
       </c>
       <c r="E7" s="13" t="s">
         <v>47</v>
@@ -27052,10 +27200,10 @@
         <v>5</v>
       </c>
       <c r="H7" s="13" t="s">
-        <v>468</v>
+        <v>517</v>
       </c>
       <c r="I7" s="13" t="s">
-        <v>469</v>
+        <v>518</v>
       </c>
       <c r="J7" s="13" t="s">
         <v>18</v>
@@ -27064,10 +27212,10 @@
         <v>47</v>
       </c>
       <c r="L7" s="13" t="s">
-        <v>470</v>
+        <v>519</v>
       </c>
       <c r="M7" s="13" t="s">
-        <v>471</v>
+        <v>520</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27078,25 +27226,25 @@
         <v>19</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>472</v>
+        <v>521</v>
       </c>
       <c r="E8" s="13" t="s">
         <v>48</v>
       </c>
       <c r="I8" s="13" t="s">
-        <v>473</v>
+        <v>522</v>
       </c>
       <c r="J8" s="13" t="s">
         <v>19</v>
       </c>
       <c r="K8" s="13" t="s">
-        <v>474</v>
+        <v>523</v>
       </c>
       <c r="L8" s="13" t="s">
-        <v>475</v>
+        <v>524</v>
       </c>
       <c r="M8" s="13" t="s">
-        <v>476</v>
+        <v>525</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27107,19 +27255,19 @@
         <v>68</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>461</v>
+        <v>510</v>
       </c>
       <c r="I9" s="13" t="s">
-        <v>477</v>
+        <v>526</v>
       </c>
       <c r="J9" s="13" t="s">
         <v>68</v>
       </c>
       <c r="L9" s="13" t="s">
-        <v>478</v>
+        <v>527</v>
       </c>
       <c r="M9" s="13" t="s">
-        <v>479</v>
+        <v>528</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27127,19 +27275,19 @@
         <v>37</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>480</v>
+        <v>529</v>
       </c>
       <c r="I10" s="13" t="s">
-        <v>481</v>
+        <v>530</v>
       </c>
       <c r="J10" s="13" t="s">
-        <v>480</v>
+        <v>529</v>
       </c>
       <c r="L10" s="13" t="s">
-        <v>482</v>
+        <v>531</v>
       </c>
       <c r="M10" s="13" t="s">
-        <v>483</v>
+        <v>532</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27147,16 +27295,16 @@
         <v>38</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>484</v>
+        <v>533</v>
       </c>
       <c r="I11" s="13" t="s">
-        <v>485</v>
+        <v>534</v>
       </c>
       <c r="L11" s="13" t="s">
         <v>39</v>
       </c>
       <c r="M11" s="13" t="s">
-        <v>486</v>
+        <v>535</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27164,38 +27312,38 @@
         <v>39</v>
       </c>
       <c r="I12" s="13" t="s">
-        <v>487</v>
+        <v>536</v>
       </c>
       <c r="M12" s="13" t="s">
-        <v>488</v>
+        <v>537</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I13" s="13" t="s">
-        <v>489</v>
+        <v>538</v>
       </c>
       <c r="M13" s="13" t="s">
-        <v>490</v>
+        <v>539</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I14" s="13" t="s">
-        <v>491</v>
+        <v>540</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I15" s="13" t="s">
-        <v>492</v>
+        <v>541</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I16" s="13" t="s">
-        <v>493</v>
+        <v>542</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I17" s="13" t="s">
-        <v>484</v>
+        <v>533</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27205,7 +27353,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I19" s="13" t="s">
-        <v>494</v>
+        <v>543</v>
       </c>
     </row>
   </sheetData>

</xml_diff>